<commit_message>
Conectar botón de licencia al backend
</commit_message>
<xml_diff>
--- a/public/docs/Ranking Catalán 2026.xlsx
+++ b/public/docs/Ranking Catalán 2026.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="58" documentId="8_{D0CAF2AB-DD7B-42E3-B202-6E1C5ACD3E1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EA83097E-A167-4543-9E26-C9ECD75B8DA6}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25180" windowHeight="16140" firstSheet="36" activeTab="41" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25180" windowHeight="16140" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Palmares" sheetId="42" r:id="rId1"/>
@@ -61,6 +61,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="33" hidden="1">'Etapa 4 Senior'!$B$2:$G$7</definedName>
   </definedNames>
   <calcPr calcId="191029" calcCompleted="0" forceFullCalc="1"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -707,7 +708,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -748,15 +749,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="5" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -2377,36 +2369,36 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{5A8ACE13-696A-4443-BA39-B9FBE82EBC6D}" name="Tabla13" displayName="Tabla13" ref="B5:Q52" totalsRowShown="0" dataDxfId="51" dataCellStyle="Normal 2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{5A8ACE13-696A-4443-BA39-B9FBE82EBC6D}" name="Tabla13" displayName="Tabla13" ref="B5:Q52" totalsRowShown="0" dataDxfId="83" dataCellStyle="Normal 2">
   <autoFilter ref="B5:Q52" xr:uid="{5A8ACE13-696A-4443-BA39-B9FBE82EBC6D}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B6:Q52">
     <sortCondition descending="1" ref="P5:P52"/>
   </sortState>
   <tableColumns count="16">
-    <tableColumn id="2" xr3:uid="{F1E38EBB-1BD8-4EE4-A3AE-ABCA3AEAC46B}" name="Posicion" dataDxfId="50" dataCellStyle="Normal 2">
+    <tableColumn id="2" xr3:uid="{F1E38EBB-1BD8-4EE4-A3AE-ABCA3AEAC46B}" name="Posicion" dataDxfId="82" dataCellStyle="Normal 2">
       <calculatedColumnFormula>ROW() - ROW($B$7) + 1</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{A1CBC385-FCC7-45A3-8079-543EE2026D15}" name="FOOTGOLFER NICKNAME" dataDxfId="49" dataCellStyle="Normal 2"/>
-    <tableColumn id="27" xr3:uid="{9D6E451B-D990-430D-B955-640E8D50D621}" name="Etapa 1" dataDxfId="48" dataCellStyle="Millares">
+    <tableColumn id="3" xr3:uid="{A1CBC385-FCC7-45A3-8079-543EE2026D15}" name="FOOTGOLFER NICKNAME" dataDxfId="81" dataCellStyle="Normal 2"/>
+    <tableColumn id="27" xr3:uid="{9D6E451B-D990-430D-B955-640E8D50D621}" name="Etapa 1" dataDxfId="80" dataCellStyle="Millares">
       <calculatedColumnFormula>IFERROR(VLOOKUP($C6,'Etapa 1 Masculino'!$E$3:$G$99,3,FALSE),0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="1" xr3:uid="{90ECDE70-1B8C-49EC-B656-CA7601ACAAF8}" name="Etapa 2" dataDxfId="47" dataCellStyle="Millares">
+    <tableColumn id="1" xr3:uid="{90ECDE70-1B8C-49EC-B656-CA7601ACAAF8}" name="Etapa 2" dataDxfId="79" dataCellStyle="Millares">
       <calculatedColumnFormula>IFERROR(VLOOKUP($C6,'Etapa 2 Masculina'!$E$3:$G$99,3,FALSE),0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{668CAF3A-214F-49B0-A7E1-07AEC7CA6CF8}" name="Etapa 3" dataDxfId="46" dataCellStyle="Millares"/>
-    <tableColumn id="5" xr3:uid="{88B5246B-EFC2-4889-A0C5-605D29DDFE2C}" name="Etapa 4" dataDxfId="45" dataCellStyle="Millares"/>
-    <tableColumn id="6" xr3:uid="{885F64CC-9069-40BA-929A-E08ADCB0198B}" name="Etapa 5" dataDxfId="44" dataCellStyle="Millares"/>
-    <tableColumn id="7" xr3:uid="{6C3E8087-8DB0-48B4-9E77-4D881811D45B}" name="Etapa 6" dataDxfId="43" dataCellStyle="Millares"/>
-    <tableColumn id="8" xr3:uid="{C7AE5939-3EE7-48F4-9206-9EA282A22377}" name="Etapa 7" dataDxfId="42" dataCellStyle="Millares"/>
-    <tableColumn id="9" xr3:uid="{4D128BD7-5B1D-4EAA-928D-A74E8508FD6C}" name="Etapa 8" dataDxfId="41" dataCellStyle="Millares"/>
-    <tableColumn id="10" xr3:uid="{BF1DEBF5-3534-4E55-85D9-BE8BD1E4C155}" name="Etapa 9" dataDxfId="40" dataCellStyle="Millares"/>
-    <tableColumn id="11" xr3:uid="{792BA664-C178-423B-A8F6-432C1F2072E7}" name="Etapa 10" dataDxfId="39" dataCellStyle="Millares"/>
-    <tableColumn id="14" xr3:uid="{6D76C7C6-EF01-41ED-9B4A-4561D0BD7544}" name="Etapa 11" dataDxfId="38" dataCellStyle="Millares"/>
-    <tableColumn id="15" xr3:uid="{AE55A304-FE5A-48C7-A282-94A30AFFAD00}" name="Etapa 12" dataDxfId="37" dataCellStyle="Millares"/>
-    <tableColumn id="12" xr3:uid="{FCD3FE0E-4A65-4CD9-A0C1-70CA31B94170}" name="Total" dataDxfId="36" dataCellStyle="Millares">
+    <tableColumn id="4" xr3:uid="{668CAF3A-214F-49B0-A7E1-07AEC7CA6CF8}" name="Etapa 3" dataDxfId="78" dataCellStyle="Millares"/>
+    <tableColumn id="5" xr3:uid="{88B5246B-EFC2-4889-A0C5-605D29DDFE2C}" name="Etapa 4" dataDxfId="77" dataCellStyle="Millares"/>
+    <tableColumn id="6" xr3:uid="{885F64CC-9069-40BA-929A-E08ADCB0198B}" name="Etapa 5" dataDxfId="76" dataCellStyle="Millares"/>
+    <tableColumn id="7" xr3:uid="{6C3E8087-8DB0-48B4-9E77-4D881811D45B}" name="Etapa 6" dataDxfId="75" dataCellStyle="Millares"/>
+    <tableColumn id="8" xr3:uid="{C7AE5939-3EE7-48F4-9206-9EA282A22377}" name="Etapa 7" dataDxfId="74" dataCellStyle="Millares"/>
+    <tableColumn id="9" xr3:uid="{4D128BD7-5B1D-4EAA-928D-A74E8508FD6C}" name="Etapa 8" dataDxfId="73" dataCellStyle="Millares"/>
+    <tableColumn id="10" xr3:uid="{BF1DEBF5-3534-4E55-85D9-BE8BD1E4C155}" name="Etapa 9" dataDxfId="72" dataCellStyle="Millares"/>
+    <tableColumn id="11" xr3:uid="{792BA664-C178-423B-A8F6-432C1F2072E7}" name="Etapa 10" dataDxfId="71" dataCellStyle="Millares"/>
+    <tableColumn id="14" xr3:uid="{6D76C7C6-EF01-41ED-9B4A-4561D0BD7544}" name="Etapa 11" dataDxfId="70" dataCellStyle="Millares"/>
+    <tableColumn id="15" xr3:uid="{AE55A304-FE5A-48C7-A282-94A30AFFAD00}" name="Etapa 12" dataDxfId="69" dataCellStyle="Millares"/>
+    <tableColumn id="12" xr3:uid="{FCD3FE0E-4A65-4CD9-A0C1-70CA31B94170}" name="Total" dataDxfId="68" dataCellStyle="Millares">
       <calculatedColumnFormula array="1">SUM(LARGE(D6:O6,{1;2;3;4;5;6;7;8}))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{028C081B-E6E0-41A7-8A9C-966CB053AB38}" name="Maxima puntuacion posible" dataDxfId="35" dataCellStyle="Normal 2">
+    <tableColumn id="13" xr3:uid="{028C081B-E6E0-41A7-8A9C-966CB053AB38}" name="Maxima puntuacion posible" dataDxfId="67" dataCellStyle="Normal 2">
       <calculatedColumnFormula array="1">SUM(LARGE(CHOOSE({1,2,3,4,5,6,7,8,9,10}, D6, E6, F6, G6, H6, I6, J6, K6, L6, 250), {1,2,3,4,5,6,7}))</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2415,36 +2407,36 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{8EC204F7-CC6F-4709-AC0C-CEFDF853C60C}" name="Tabla139" displayName="Tabla139" ref="B5:Q49" totalsRowShown="0" dataDxfId="34" dataCellStyle="Normal 2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{8EC204F7-CC6F-4709-AC0C-CEFDF853C60C}" name="Tabla139" displayName="Tabla139" ref="B5:Q49" totalsRowShown="0" dataDxfId="51" dataCellStyle="Normal 2">
   <autoFilter ref="B5:Q49" xr:uid="{8EC204F7-CC6F-4709-AC0C-CEFDF853C60C}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B6:Q49">
     <sortCondition descending="1" ref="P5:P49"/>
   </sortState>
   <tableColumns count="16">
-    <tableColumn id="2" xr3:uid="{30A85A4E-EEFB-4FF5-930E-F7B30744104E}" name="Posicion" dataDxfId="33" dataCellStyle="Normal 2">
+    <tableColumn id="2" xr3:uid="{30A85A4E-EEFB-4FF5-930E-F7B30744104E}" name="Posicion" dataDxfId="50" dataCellStyle="Normal 2">
       <calculatedColumnFormula>ROW() - ROW($B$6) + 1</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{3C3D434E-7585-4D95-8296-D1E67234ECB8}" name="FOOTGOLFER NICKNAME" dataDxfId="32" dataCellStyle="Normal 2"/>
-    <tableColumn id="27" xr3:uid="{CDB33A2E-57AA-4478-923B-058E0904A198}" name="Etapa 1" dataDxfId="31" dataCellStyle="Millares">
+    <tableColumn id="3" xr3:uid="{3C3D434E-7585-4D95-8296-D1E67234ECB8}" name="FOOTGOLFER NICKNAME" dataDxfId="49" dataCellStyle="Normal 2"/>
+    <tableColumn id="27" xr3:uid="{CDB33A2E-57AA-4478-923B-058E0904A198}" name="Etapa 1" dataDxfId="48" dataCellStyle="Millares">
       <calculatedColumnFormula>IFERROR(VLOOKUP($C6,'Etapa 1 Senior'!$E$3:$G$83,3,FALSE),0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="1" xr3:uid="{4AC31F12-1D47-4E5B-B342-93C496635CEC}" name="Etapa 2" dataDxfId="30" dataCellStyle="Millares">
+    <tableColumn id="1" xr3:uid="{4AC31F12-1D47-4E5B-B342-93C496635CEC}" name="Etapa 2" dataDxfId="47" dataCellStyle="Millares">
       <calculatedColumnFormula>IFERROR(VLOOKUP($C6,'Etapa 2 Senior'!$E$3:$G$83,3,FALSE),0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{C25FCC5D-8058-4E0D-A1A7-288B76F84A2C}" name="Etapa 3" dataDxfId="29" dataCellStyle="Millares"/>
-    <tableColumn id="5" xr3:uid="{651C490E-9B92-4DDC-A1BD-AB93B8B9E0AD}" name="Etapa 4" dataDxfId="28" dataCellStyle="Millares"/>
-    <tableColumn id="6" xr3:uid="{F8F451D1-AE51-4400-84DA-8DF60622FB45}" name="Etapa 5" dataDxfId="27" dataCellStyle="Millares"/>
-    <tableColumn id="7" xr3:uid="{12D2A034-DFCB-499E-8930-08DD7BB8BE61}" name="Etapa 6" dataDxfId="26" dataCellStyle="Millares"/>
-    <tableColumn id="8" xr3:uid="{E7D2D98B-6F18-499F-9E5D-ABBA9D22AEBE}" name="Etapa 7" dataDxfId="25" dataCellStyle="Millares"/>
-    <tableColumn id="9" xr3:uid="{058962A3-8B6D-4686-8B78-7BFDF5815A2D}" name="Etapa 8" dataDxfId="24" dataCellStyle="Millares"/>
-    <tableColumn id="10" xr3:uid="{4BE3F3FE-B622-468E-9BCF-6BF978CEAB53}" name="Etapa 9" dataDxfId="23" dataCellStyle="Millares"/>
-    <tableColumn id="11" xr3:uid="{3EF8476E-0FD4-4648-9890-9094D2BF4514}" name="Etapa 10" dataDxfId="22" dataCellStyle="Millares"/>
-    <tableColumn id="14" xr3:uid="{72F9CADB-7B95-4EED-8F4E-29427821D2EB}" name="Etapa 11" dataDxfId="21" dataCellStyle="Millares"/>
-    <tableColumn id="15" xr3:uid="{D3302936-8031-4F4B-A334-52A32696E49D}" name="Etapa 12" dataDxfId="20" dataCellStyle="Millares"/>
-    <tableColumn id="12" xr3:uid="{4EA1A9BD-6347-48F9-97EC-82D1BBF11FF3}" name="Total" dataDxfId="19" dataCellStyle="Millares">
+    <tableColumn id="4" xr3:uid="{C25FCC5D-8058-4E0D-A1A7-288B76F84A2C}" name="Etapa 3" dataDxfId="46" dataCellStyle="Millares"/>
+    <tableColumn id="5" xr3:uid="{651C490E-9B92-4DDC-A1BD-AB93B8B9E0AD}" name="Etapa 4" dataDxfId="45" dataCellStyle="Millares"/>
+    <tableColumn id="6" xr3:uid="{F8F451D1-AE51-4400-84DA-8DF60622FB45}" name="Etapa 5" dataDxfId="44" dataCellStyle="Millares"/>
+    <tableColumn id="7" xr3:uid="{12D2A034-DFCB-499E-8930-08DD7BB8BE61}" name="Etapa 6" dataDxfId="43" dataCellStyle="Millares"/>
+    <tableColumn id="8" xr3:uid="{E7D2D98B-6F18-499F-9E5D-ABBA9D22AEBE}" name="Etapa 7" dataDxfId="42" dataCellStyle="Millares"/>
+    <tableColumn id="9" xr3:uid="{058962A3-8B6D-4686-8B78-7BFDF5815A2D}" name="Etapa 8" dataDxfId="41" dataCellStyle="Millares"/>
+    <tableColumn id="10" xr3:uid="{4BE3F3FE-B622-468E-9BCF-6BF978CEAB53}" name="Etapa 9" dataDxfId="40" dataCellStyle="Millares"/>
+    <tableColumn id="11" xr3:uid="{3EF8476E-0FD4-4648-9890-9094D2BF4514}" name="Etapa 10" dataDxfId="39" dataCellStyle="Millares"/>
+    <tableColumn id="14" xr3:uid="{72F9CADB-7B95-4EED-8F4E-29427821D2EB}" name="Etapa 11" dataDxfId="38" dataCellStyle="Millares"/>
+    <tableColumn id="15" xr3:uid="{D3302936-8031-4F4B-A334-52A32696E49D}" name="Etapa 12" dataDxfId="37" dataCellStyle="Millares"/>
+    <tableColumn id="12" xr3:uid="{4EA1A9BD-6347-48F9-97EC-82D1BBF11FF3}" name="Total" dataDxfId="36" dataCellStyle="Millares">
       <calculatedColumnFormula array="1">SUM(LARGE(D6:O6,{1;2;3;4;5;6;7;8}))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{A0AEBCBB-ECB8-44A6-998D-C63842DADC41}" name="Maxima puntuacion posible" dataDxfId="18" dataCellStyle="Normal 2">
+    <tableColumn id="13" xr3:uid="{A0AEBCBB-ECB8-44A6-998D-C63842DADC41}" name="Maxima puntuacion posible" dataDxfId="35" dataCellStyle="Normal 2">
       <calculatedColumnFormula array="1">SUM(LARGE(CHOOSE({1,2,3,4,5,6,7,8,9,10}, D6, E6, F6, G6, H6, I6, J6, K6, L6, 250), {1,2,3,4,5,6,7}))</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2453,36 +2445,36 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{6E9802BB-9A96-44D1-8C01-C250B3B7B656}" name="Tabla13911" displayName="Tabla13911" ref="B5:Q52" totalsRowShown="0" dataDxfId="83" dataCellStyle="Normal 2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{6E9802BB-9A96-44D1-8C01-C250B3B7B656}" name="Tabla13911" displayName="Tabla13911" ref="B5:Q52" totalsRowShown="0" dataDxfId="34" dataCellStyle="Normal 2">
   <autoFilter ref="B5:Q52" xr:uid="{6E9802BB-9A96-44D1-8C01-C250B3B7B656}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B6:Q52">
     <sortCondition descending="1" ref="P5:P52"/>
   </sortState>
   <tableColumns count="16">
-    <tableColumn id="2" xr3:uid="{892EA637-6C36-42DD-8D6E-9221B98768F1}" name="Posicion" dataDxfId="82" dataCellStyle="Normal 2">
+    <tableColumn id="2" xr3:uid="{892EA637-6C36-42DD-8D6E-9221B98768F1}" name="Posicion" dataDxfId="33" dataCellStyle="Normal 2">
       <calculatedColumnFormula>ROW() - ROW($B$7) + 1</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{9716F7C5-ED1A-4435-992D-5FB49F1ED6CB}" name="FOOTGOLFER NICKNAME" dataDxfId="81" dataCellStyle="Normal 2"/>
-    <tableColumn id="27" xr3:uid="{F5476534-2D61-472E-80D0-C1D79689B28A}" name="Etapa 1" dataDxfId="80" dataCellStyle="Millares">
+    <tableColumn id="3" xr3:uid="{9716F7C5-ED1A-4435-992D-5FB49F1ED6CB}" name="FOOTGOLFER NICKNAME" dataDxfId="32" dataCellStyle="Normal 2"/>
+    <tableColumn id="27" xr3:uid="{F5476534-2D61-472E-80D0-C1D79689B28A}" name="Etapa 1" dataDxfId="31" dataCellStyle="Millares">
       <calculatedColumnFormula>IFERROR(VLOOKUP($C6,'Etapa 1 Rookie'!$E$3:$G$83,3,FALSE),0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="1" xr3:uid="{C41457E1-3203-4775-AC35-550B3EDDE18A}" name="Etapa 2" dataDxfId="79" dataCellStyle="Millares">
+    <tableColumn id="1" xr3:uid="{C41457E1-3203-4775-AC35-550B3EDDE18A}" name="Etapa 2" dataDxfId="30" dataCellStyle="Millares">
       <calculatedColumnFormula>IFERROR(VLOOKUP($C6,'Etapa 2 Rookie'!$E$3:$G$83,3,FALSE),0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{80F89B60-247C-49FA-B598-39D89905D8E9}" name="Etapa 3" dataDxfId="78" dataCellStyle="Millares"/>
-    <tableColumn id="5" xr3:uid="{3F35F293-8DB3-41A0-AF8A-FDE7830D3664}" name="Etapa 4" dataDxfId="77" dataCellStyle="Millares"/>
-    <tableColumn id="6" xr3:uid="{993F21BB-1247-442A-8A83-43F0667F1A71}" name="Etapa 5" dataDxfId="76" dataCellStyle="Millares"/>
-    <tableColumn id="7" xr3:uid="{1F403493-6E22-4254-9703-824E3DA8521A}" name="Etapa 6" dataDxfId="75" dataCellStyle="Millares"/>
-    <tableColumn id="8" xr3:uid="{57634BDF-F17E-4FCA-88E0-874363FEDC46}" name="Etapa 7" dataDxfId="74" dataCellStyle="Millares"/>
-    <tableColumn id="9" xr3:uid="{96A382FC-9F8C-4BD7-A55C-75C3C3EAAF56}" name="Etapa 8" dataDxfId="73" dataCellStyle="Millares"/>
-    <tableColumn id="10" xr3:uid="{A287AE7E-6A5B-42B0-ACD9-796094E34063}" name="Etapa 9" dataDxfId="72" dataCellStyle="Millares"/>
-    <tableColumn id="11" xr3:uid="{0BCE5D5B-CFAC-49C6-9B92-9D4DF75FF5FD}" name="Etapa 10" dataDxfId="71" dataCellStyle="Millares"/>
-    <tableColumn id="14" xr3:uid="{2310C24A-B92E-4FA0-9160-BEE144CA8369}" name="Etapa 11" dataDxfId="70" dataCellStyle="Millares"/>
-    <tableColumn id="15" xr3:uid="{F5CEEC85-5388-4DC1-9BD9-B7826E8BE188}" name="Etapa 12" dataDxfId="69" dataCellStyle="Millares"/>
-    <tableColumn id="12" xr3:uid="{CFA4579C-3142-4F51-932F-C910E2104ABB}" name="Total" dataDxfId="68" dataCellStyle="Millares">
+    <tableColumn id="4" xr3:uid="{80F89B60-247C-49FA-B598-39D89905D8E9}" name="Etapa 3" dataDxfId="29" dataCellStyle="Millares"/>
+    <tableColumn id="5" xr3:uid="{3F35F293-8DB3-41A0-AF8A-FDE7830D3664}" name="Etapa 4" dataDxfId="28" dataCellStyle="Millares"/>
+    <tableColumn id="6" xr3:uid="{993F21BB-1247-442A-8A83-43F0667F1A71}" name="Etapa 5" dataDxfId="27" dataCellStyle="Millares"/>
+    <tableColumn id="7" xr3:uid="{1F403493-6E22-4254-9703-824E3DA8521A}" name="Etapa 6" dataDxfId="26" dataCellStyle="Millares"/>
+    <tableColumn id="8" xr3:uid="{57634BDF-F17E-4FCA-88E0-874363FEDC46}" name="Etapa 7" dataDxfId="25" dataCellStyle="Millares"/>
+    <tableColumn id="9" xr3:uid="{96A382FC-9F8C-4BD7-A55C-75C3C3EAAF56}" name="Etapa 8" dataDxfId="24" dataCellStyle="Millares"/>
+    <tableColumn id="10" xr3:uid="{A287AE7E-6A5B-42B0-ACD9-796094E34063}" name="Etapa 9" dataDxfId="23" dataCellStyle="Millares"/>
+    <tableColumn id="11" xr3:uid="{0BCE5D5B-CFAC-49C6-9B92-9D4DF75FF5FD}" name="Etapa 10" dataDxfId="22" dataCellStyle="Millares"/>
+    <tableColumn id="14" xr3:uid="{2310C24A-B92E-4FA0-9160-BEE144CA8369}" name="Etapa 11" dataDxfId="21" dataCellStyle="Millares"/>
+    <tableColumn id="15" xr3:uid="{F5CEEC85-5388-4DC1-9BD9-B7826E8BE188}" name="Etapa 12" dataDxfId="20" dataCellStyle="Millares"/>
+    <tableColumn id="12" xr3:uid="{CFA4579C-3142-4F51-932F-C910E2104ABB}" name="Total" dataDxfId="19" dataCellStyle="Millares">
       <calculatedColumnFormula array="1">SUM(LARGE(D6:O6,{1;2;3;4;5;6;7;8}))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{D2B0A136-E6A3-491C-BD06-B9A7F1C5C376}" name="Maxima puntuacion posible" dataDxfId="67" dataCellStyle="Normal 2">
+    <tableColumn id="13" xr3:uid="{D2B0A136-E6A3-491C-BD06-B9A7F1C5C376}" name="Maxima puntuacion posible" dataDxfId="18" dataCellStyle="Normal 2">
       <calculatedColumnFormula array="1">SUM(LARGE(CHOOSE({1,2,3,4,5,6,7,8,9,10}, D6, E6, F6, G6, H6, I6, J6, K6, L6, 250), {1,2,3,4,5,6,7}))</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -14251,7 +14243,7 @@
         <f t="shared" si="0"/>
         <v>23</v>
       </c>
-      <c r="C28" s="17" t="s">
+      <c r="C28" s="6" t="s">
         <v>143</v>
       </c>
       <c r="D28" s="7">
@@ -14292,11 +14284,11 @@
       <c r="O28" s="7">
         <v>0</v>
       </c>
-      <c r="P28" s="18" cm="1">
+      <c r="P28" s="7" cm="1">
         <f t="array" ref="P28">SUM(LARGE(D28:O28,{1;2;3;4;5;6;7;8}))</f>
         <v>92.5</v>
       </c>
-      <c r="Q28" s="19" cm="1">
+      <c r="Q28" s="6" cm="1">
         <f t="array" ref="Q28">SUM(LARGE(CHOOSE({1,2,3,4,5,6,7,8,9,10}, D28, E28, F28, G28, H28, I28, J28, K28, L28, 250), {1,2,3,4,5,6,7}))</f>
         <v>342.5</v>
       </c>
@@ -14361,7 +14353,7 @@
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
-      <c r="C30" s="17" t="s">
+      <c r="C30" s="6" t="s">
         <v>144</v>
       </c>
       <c r="D30" s="7">
@@ -14402,11 +14394,11 @@
       <c r="O30" s="7">
         <v>0</v>
       </c>
-      <c r="P30" s="18" cm="1">
+      <c r="P30" s="7" cm="1">
         <f t="array" ref="P30">SUM(LARGE(D30:O30,{1;2;3;4;5;6;7;8}))</f>
         <v>75</v>
       </c>
-      <c r="Q30" s="19" cm="1">
+      <c r="Q30" s="6" cm="1">
         <f t="array" ref="Q30">SUM(LARGE(CHOOSE({1,2,3,4,5,6,7,8,9,10}, D30, E30, F30, G30, H30, I30, J30, K30, L30, 250), {1,2,3,4,5,6,7}))</f>
         <v>325</v>
       </c>
@@ -18151,7 +18143,7 @@
     </row>
     <row r="6" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B6">
-        <f>COUNTIFS($F$3:$F$996,"&lt;"&amp;$F6)+1</f>
+        <f t="shared" ref="B6:B24" si="0">COUNTIFS($F$3:$F$996,"&lt;"&amp;$F6)+1</f>
         <v>2</v>
       </c>
       <c r="C6" t="s">
@@ -18180,7 +18172,7 @@
     </row>
     <row r="7" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B7">
-        <f>COUNTIFS($F$3:$F$996,"&lt;"&amp;$F7)+1</f>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="C7" t="s">
@@ -18209,7 +18201,7 @@
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B8">
-        <f>COUNTIFS($F$3:$F$996,"&lt;"&amp;$F8)+1</f>
+        <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="C8" t="s">
@@ -18238,7 +18230,7 @@
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B9">
-        <f>COUNTIFS($F$3:$F$996,"&lt;"&amp;$F9)+1</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="C9" t="s">
@@ -18267,7 +18259,7 @@
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B10">
-        <f>COUNTIFS($F$3:$F$996,"&lt;"&amp;$F10)+1</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="C10" t="s">
@@ -18296,7 +18288,7 @@
     </row>
     <row r="11" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B11">
-        <f>COUNTIFS($F$3:$F$996,"&lt;"&amp;$F11)+1</f>
+        <f t="shared" si="0"/>
         <v>9</v>
       </c>
       <c r="C11" t="s">
@@ -18325,7 +18317,7 @@
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B12">
-        <f>COUNTIFS($F$3:$F$996,"&lt;"&amp;$F12)+1</f>
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="C12" t="s">
@@ -18354,7 +18346,7 @@
     </row>
     <row r="13" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B13">
-        <f>COUNTIFS($F$3:$F$996,"&lt;"&amp;$F13)+1</f>
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
       <c r="C13" t="s">
@@ -18383,7 +18375,7 @@
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B14">
-        <f>COUNTIFS($F$3:$F$996,"&lt;"&amp;$F14)+1</f>
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
       <c r="C14" t="s">
@@ -18412,7 +18404,7 @@
     </row>
     <row r="15" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B15">
-        <f>COUNTIFS($F$3:$F$996,"&lt;"&amp;$F15)+1</f>
+        <f t="shared" si="0"/>
         <v>13</v>
       </c>
       <c r="C15" t="s">
@@ -18441,7 +18433,7 @@
     </row>
     <row r="16" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B16">
-        <f>COUNTIFS($F$3:$F$996,"&lt;"&amp;$F16)+1</f>
+        <f t="shared" si="0"/>
         <v>14</v>
       </c>
       <c r="C16" t="s">
@@ -18470,7 +18462,7 @@
     </row>
     <row r="17" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B17">
-        <f>COUNTIFS($F$3:$F$996,"&lt;"&amp;$F17)+1</f>
+        <f t="shared" si="0"/>
         <v>15</v>
       </c>
       <c r="C17" t="s">
@@ -18499,7 +18491,7 @@
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B18">
-        <f>COUNTIFS($F$3:$F$996,"&lt;"&amp;$F18)+1</f>
+        <f t="shared" si="0"/>
         <v>15</v>
       </c>
       <c r="C18" t="s">
@@ -18528,7 +18520,7 @@
     </row>
     <row r="19" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B19">
-        <f>COUNTIFS($F$3:$F$996,"&lt;"&amp;$F19)+1</f>
+        <f t="shared" si="0"/>
         <v>17</v>
       </c>
       <c r="C19" t="s">
@@ -18557,7 +18549,7 @@
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B20">
-        <f>COUNTIFS($F$3:$F$996,"&lt;"&amp;$F20)+1</f>
+        <f t="shared" si="0"/>
         <v>18</v>
       </c>
       <c r="C20" t="s">
@@ -18586,7 +18578,7 @@
     </row>
     <row r="21" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B21">
-        <f>COUNTIFS($F$3:$F$996,"&lt;"&amp;$F21)+1</f>
+        <f t="shared" si="0"/>
         <v>19</v>
       </c>
       <c r="C21" t="s">
@@ -18615,7 +18607,7 @@
     </row>
     <row r="22" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B22">
-        <f>COUNTIFS($F$3:$F$996,"&lt;"&amp;$F22)+1</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="C22" t="s">
@@ -18644,7 +18636,7 @@
     </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B23">
-        <f>COUNTIFS($F$3:$F$996,"&lt;"&amp;$F23)+1</f>
+        <f t="shared" si="0"/>
         <v>21</v>
       </c>
       <c r="C23" t="s">
@@ -18673,7 +18665,7 @@
     </row>
     <row r="24" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B24">
-        <f>COUNTIFS($F$3:$F$996,"&lt;"&amp;$F24)+1</f>
+        <f t="shared" si="0"/>
         <v>22</v>
       </c>
       <c r="C24" t="s">
@@ -18743,7 +18735,7 @@
     </row>
     <row r="3" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B3">
-        <f>COUNTIFS($F$3:$F$980,"&lt;"&amp;$F3)+1</f>
+        <f t="shared" ref="B3:B8" si="0">COUNTIFS($F$3:$F$980,"&lt;"&amp;$F3)+1</f>
         <v>1</v>
       </c>
       <c r="C3" t="s">
@@ -18772,7 +18764,7 @@
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B4">
-        <f>COUNTIFS($F$3:$F$980,"&lt;"&amp;$F4)+1</f>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="C4" t="s">
@@ -18801,7 +18793,7 @@
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B5">
-        <f>COUNTIFS($F$3:$F$980,"&lt;"&amp;$F5)+1</f>
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="C5" t="s">
@@ -18830,7 +18822,7 @@
     </row>
     <row r="6" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B6">
-        <f>COUNTIFS($F$3:$F$980,"&lt;"&amp;$F6)+1</f>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="C6" t="s">
@@ -18859,7 +18851,7 @@
     </row>
     <row r="7" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B7">
-        <f>COUNTIFS($F$3:$F$980,"&lt;"&amp;$F7)+1</f>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="C7" t="s">
@@ -18888,7 +18880,7 @@
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B8">
-        <f>COUNTIFS($F$3:$F$980,"&lt;"&amp;$F8)+1</f>
+        <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="C8" t="s">
@@ -18983,7 +18975,7 @@
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B4">
-        <f>COUNTIFS($F$3:$F$989,"&lt;"&amp;$F4)+1</f>
+        <f t="shared" ref="B4:B17" si="0">COUNTIFS($F$3:$F$989,"&lt;"&amp;$F4)+1</f>
         <v>1</v>
       </c>
       <c r="C4" t="s">
@@ -19012,7 +19004,7 @@
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B5">
-        <f>COUNTIFS($F$3:$F$989,"&lt;"&amp;$F5)+1</f>
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="C5" t="s">
@@ -19041,7 +19033,7 @@
     </row>
     <row r="6" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B6">
-        <f>COUNTIFS($F$3:$F$989,"&lt;"&amp;$F6)+1</f>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="C6" t="s">
@@ -19070,7 +19062,7 @@
     </row>
     <row r="7" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B7">
-        <f>COUNTIFS($F$3:$F$989,"&lt;"&amp;$F7)+1</f>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="C7" t="s">
@@ -19099,7 +19091,7 @@
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B8">
-        <f>COUNTIFS($F$3:$F$989,"&lt;"&amp;$F8)+1</f>
+        <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="C8" t="s">
@@ -19128,7 +19120,7 @@
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B9">
-        <f>COUNTIFS($F$3:$F$989,"&lt;"&amp;$F9)+1</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="C9" t="s">
@@ -19157,7 +19149,7 @@
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B10">
-        <f>COUNTIFS($F$3:$F$989,"&lt;"&amp;$F10)+1</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="C10" t="s">
@@ -19186,7 +19178,7 @@
     </row>
     <row r="11" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B11">
-        <f>COUNTIFS($F$3:$F$989,"&lt;"&amp;$F11)+1</f>
+        <f t="shared" si="0"/>
         <v>9</v>
       </c>
       <c r="C11" t="s">
@@ -19215,7 +19207,7 @@
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B12">
-        <f>COUNTIFS($F$3:$F$989,"&lt;"&amp;$F12)+1</f>
+        <f t="shared" si="0"/>
         <v>9</v>
       </c>
       <c r="C12" t="s">
@@ -19244,7 +19236,7 @@
     </row>
     <row r="13" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B13">
-        <f>COUNTIFS($F$3:$F$989,"&lt;"&amp;$F13)+1</f>
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
       <c r="C13" t="s">
@@ -19273,7 +19265,7 @@
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B14">
-        <f>COUNTIFS($F$3:$F$989,"&lt;"&amp;$F14)+1</f>
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
       <c r="C14" t="s">
@@ -19302,7 +19294,7 @@
     </row>
     <row r="15" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B15">
-        <f>COUNTIFS($F$3:$F$989,"&lt;"&amp;$F15)+1</f>
+        <f t="shared" si="0"/>
         <v>13</v>
       </c>
       <c r="C15" t="s">
@@ -19331,7 +19323,7 @@
     </row>
     <row r="16" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B16">
-        <f>COUNTIFS($F$3:$F$989,"&lt;"&amp;$F16)+1</f>
+        <f t="shared" si="0"/>
         <v>14</v>
       </c>
       <c r="C16" t="s">
@@ -19360,7 +19352,7 @@
     </row>
     <row r="17" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B17">
-        <f>COUNTIFS($F$3:$F$989,"&lt;"&amp;$F17)+1</f>
+        <f t="shared" si="0"/>
         <v>15</v>
       </c>
       <c r="C17" t="s">
@@ -24547,7 +24539,7 @@
     </row>
     <row r="6" spans="2:22" ht="18.5" x14ac:dyDescent="0.45">
       <c r="B6" s="6">
-        <f>ROW() - ROW($B$6) + 1</f>
+        <f t="shared" ref="B6:B11" si="0">ROW() - ROW($B$6) + 1</f>
         <v>1</v>
       </c>
       <c r="C6" s="6" t="s">
@@ -24608,7 +24600,7 @@
     </row>
     <row r="7" spans="2:22" ht="18.5" x14ac:dyDescent="0.45">
       <c r="B7" s="6">
-        <f>ROW() - ROW($B$6) + 1</f>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="C7" s="6" t="s">
@@ -24669,7 +24661,7 @@
     </row>
     <row r="8" spans="2:22" ht="18.5" x14ac:dyDescent="0.45">
       <c r="B8" s="6">
-        <f>ROW() - ROW($B$6) + 1</f>
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="C8" s="6" t="s">
@@ -24730,7 +24722,7 @@
     </row>
     <row r="9" spans="2:22" ht="18.5" x14ac:dyDescent="0.45">
       <c r="B9" s="6">
-        <f>ROW() - ROW($B$6) + 1</f>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="C9" s="6" t="s">
@@ -24785,7 +24777,7 @@
     </row>
     <row r="10" spans="2:22" ht="18.5" x14ac:dyDescent="0.45">
       <c r="B10" s="6">
-        <f>ROW() - ROW($B$6) + 1</f>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="C10" s="6" t="s">
@@ -24840,7 +24832,7 @@
     </row>
     <row r="11" spans="2:22" ht="18.5" x14ac:dyDescent="0.45">
       <c r="B11" s="6">
-        <f>ROW() - ROW($B$6) + 1</f>
+        <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="C11" s="6" t="s">
@@ -25330,11 +25322,11 @@
       </c>
     </row>
     <row r="20" spans="2:17" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="B20" s="17">
+      <c r="B20" s="6">
         <f>ROW() - ROW($B$7) + 1</f>
         <v>14</v>
       </c>
-      <c r="C20" s="17" t="s">
+      <c r="C20" s="6" t="s">
         <v>143</v>
       </c>
       <c r="D20" s="7">
@@ -25375,21 +25367,21 @@
       <c r="O20" s="7">
         <v>0</v>
       </c>
-      <c r="P20" s="18" cm="1">
+      <c r="P20" s="7" cm="1">
         <f t="array" ref="P20">SUM(LARGE(D20:O20,{1;2;3;4;5;6;7;8}))</f>
         <v>145</v>
       </c>
-      <c r="Q20" s="19" cm="1">
+      <c r="Q20" s="6" cm="1">
         <f t="array" ref="Q20">SUM(LARGE(CHOOSE({1,2,3,4,5,6,7,8,9,10}, D20, E20, F20, G20, H20, I20, J20, K20, L20, 250), {1,2,3,4,5,6,7}))</f>
         <v>395</v>
       </c>
     </row>
     <row r="21" spans="2:17" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="B21" s="17">
+      <c r="B21" s="6">
         <f>ROW() - ROW($B$7) + 1</f>
         <v>15</v>
       </c>
-      <c r="C21" s="17" t="s">
+      <c r="C21" s="6" t="s">
         <v>144</v>
       </c>
       <c r="D21" s="7">
@@ -25430,11 +25422,11 @@
       <c r="O21" s="7">
         <v>0</v>
       </c>
-      <c r="P21" s="18" cm="1">
+      <c r="P21" s="7" cm="1">
         <f t="array" ref="P21">SUM(LARGE(D21:O21,{1;2;3;4;5;6;7;8}))</f>
         <v>110</v>
       </c>
-      <c r="Q21" s="19" cm="1">
+      <c r="Q21" s="6" cm="1">
         <f t="array" ref="Q21">SUM(LARGE(CHOOSE({1,2,3,4,5,6,7,8,9,10}, D21, E21, F21, G21, H21, I21, J21, K21, L21, 250), {1,2,3,4,5,6,7}))</f>
         <v>360</v>
       </c>
@@ -25605,7 +25597,7 @@
     </row>
     <row r="25" spans="2:17" ht="18.5" x14ac:dyDescent="0.45">
       <c r="B25" s="6">
-        <f>ROW() - ROW($B$6) + 1</f>
+        <f t="shared" ref="B25:B35" si="1">ROW() - ROW($B$6) + 1</f>
         <v>20</v>
       </c>
       <c r="C25" s="6" t="s">
@@ -25660,7 +25652,7 @@
     </row>
     <row r="26" spans="2:17" ht="18.5" x14ac:dyDescent="0.45">
       <c r="B26" s="6">
-        <f>ROW() - ROW($B$6) + 1</f>
+        <f t="shared" si="1"/>
         <v>21</v>
       </c>
       <c r="C26" s="6" t="s">
@@ -25715,7 +25707,7 @@
     </row>
     <row r="27" spans="2:17" ht="18.5" x14ac:dyDescent="0.45">
       <c r="B27" s="6">
-        <f>ROW() - ROW($B$6) + 1</f>
+        <f t="shared" si="1"/>
         <v>22</v>
       </c>
       <c r="C27" s="6" t="s">
@@ -25770,7 +25762,7 @@
     </row>
     <row r="28" spans="2:17" ht="18.5" x14ac:dyDescent="0.45">
       <c r="B28" s="6">
-        <f>ROW() - ROW($B$6) + 1</f>
+        <f t="shared" si="1"/>
         <v>23</v>
       </c>
       <c r="C28" s="6" t="s">
@@ -25825,7 +25817,7 @@
     </row>
     <row r="29" spans="2:17" ht="18.5" x14ac:dyDescent="0.45">
       <c r="B29" s="6">
-        <f>ROW() - ROW($B$6) + 1</f>
+        <f t="shared" si="1"/>
         <v>24</v>
       </c>
       <c r="C29" s="6" t="s">
@@ -25880,7 +25872,7 @@
     </row>
     <row r="30" spans="2:17" ht="18.5" x14ac:dyDescent="0.45">
       <c r="B30" s="6">
-        <f>ROW() - ROW($B$6) + 1</f>
+        <f t="shared" si="1"/>
         <v>25</v>
       </c>
       <c r="C30" s="6" t="s">
@@ -25935,7 +25927,7 @@
     </row>
     <row r="31" spans="2:17" ht="18.5" x14ac:dyDescent="0.45">
       <c r="B31" s="6">
-        <f>ROW() - ROW($B$6) + 1</f>
+        <f t="shared" si="1"/>
         <v>26</v>
       </c>
       <c r="C31" s="6" t="s">
@@ -25990,7 +25982,7 @@
     </row>
     <row r="32" spans="2:17" ht="18.5" x14ac:dyDescent="0.45">
       <c r="B32" s="6">
-        <f>ROW() - ROW($B$6) + 1</f>
+        <f t="shared" si="1"/>
         <v>27</v>
       </c>
       <c r="C32" s="6" t="s">
@@ -26045,7 +26037,7 @@
     </row>
     <row r="33" spans="2:17" ht="18.5" x14ac:dyDescent="0.45">
       <c r="B33" s="6">
-        <f>ROW() - ROW($B$6) + 1</f>
+        <f t="shared" si="1"/>
         <v>28</v>
       </c>
       <c r="C33" s="6" t="s">
@@ -26100,7 +26092,7 @@
     </row>
     <row r="34" spans="2:17" ht="18.5" x14ac:dyDescent="0.45">
       <c r="B34" s="6">
-        <f>ROW() - ROW($B$6) + 1</f>
+        <f t="shared" si="1"/>
         <v>29</v>
       </c>
       <c r="C34" s="6" t="s">
@@ -26155,7 +26147,7 @@
     </row>
     <row r="35" spans="2:17" ht="18.5" x14ac:dyDescent="0.45">
       <c r="B35" s="6">
-        <f>ROW() - ROW($B$6) + 1</f>
+        <f t="shared" si="1"/>
         <v>30</v>
       </c>
       <c r="C35" s="6" t="s">

</xml_diff>

<commit_message>
Fix: logic for detailed rankings and new categories (Junior, Damas)
</commit_message>
<xml_diff>
--- a/public/docs/Ranking Catalán 2026.xlsx
+++ b/public/docs/Ranking Catalán 2026.xlsx
@@ -60,8 +60,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Etapa 1 Masculino'!$B$2:$F$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="33" hidden="1">'Etapa 4 Senior'!$B$2:$G$7</definedName>
   </definedNames>
-  <calcPr calcId="191029" calcCompleted="0" forceFullCalc="1"/>
-  <fileRecoveryPr repairLoad="1"/>
+  <calcPr calcId="191029" forceFullCalc="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -642,6 +641,7 @@
     <font>
       <sz val="8"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="9">

</xml_diff>